<commit_message>
Auto backup 2026-06-30 10:35:01
</commit_message>
<xml_diff>
--- a/SwissTechAhsan/AHSAN/OFFICE FILE.xlsx
+++ b/SwissTechAhsan/AHSAN/OFFICE FILE.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="55">
   <si>
     <t>DATE</t>
   </si>
@@ -129,9 +129,6 @@
   </si>
   <si>
     <t>GHULAM REZA JANGJO</t>
-  </si>
-  <si>
-    <t>OFFICE WORK 0601</t>
   </si>
   <si>
     <t>DUBAI ELECTRICTY</t>
@@ -554,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
@@ -773,303 +770,248 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
-        <v>46196</v>
+        <v>46179</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="3">
-        <v>5691</v>
+        <v>39</v>
+      </c>
+      <c r="C20" s="7">
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
-        <v>46196</v>
+        <v>46180</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="3">
-        <v>224.2</v>
+        <v>35</v>
+      </c>
+      <c r="C21" s="7">
+        <v>2398</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
-        <v>46196</v>
+        <v>46181</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" s="3">
-        <v>4198</v>
+        <v>38</v>
+      </c>
+      <c r="C22" s="5">
+        <v>2398</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
-        <v>46196</v>
+        <v>46181</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C23" s="3">
-        <v>236</v>
+        <v>38</v>
+      </c>
+      <c r="C23" s="5">
+        <v>2398</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
-        <v>46196</v>
+        <v>46184</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C24" s="3">
-        <v>4300</v>
+        <v>46</v>
+      </c>
+      <c r="C24" s="1">
+        <v>1130.4100000000001</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
-        <v>46179</v>
+        <v>46184</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C25" s="7">
-        <v>4.5999999999999996</v>
+        <v>47</v>
+      </c>
+      <c r="C25" s="5">
+        <v>1122</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
-        <v>46180</v>
+        <v>46194</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C26" s="7">
-        <v>2398</v>
+        <v>50</v>
+      </c>
+      <c r="C26" s="5">
+        <v>224</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
-        <v>46181</v>
+        <v>46194</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C27" s="5">
-        <v>2398</v>
+        <v>472</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
-        <v>46181</v>
+        <v>46194</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C28" s="5">
-        <v>2398</v>
+        <v>3794</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
-        <v>46184</v>
+        <v>46194</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C29" s="1">
-        <v>1130.4100000000001</v>
+        <v>51</v>
+      </c>
+      <c r="C29" s="5">
+        <v>570</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
-        <v>46184</v>
+        <v>46195</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C30" s="5">
-        <v>1122</v>
+        <v>3912</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C31" s="5">
-        <v>224</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C32" s="5">
-        <v>472</v>
+        <v>590</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
-        <v>46194</v>
+        <v>46196</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C33" s="5">
-        <v>3794</v>
+      <c r="C33" s="7">
+        <v>4300</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
-        <v>46194</v>
+        <v>46196</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C34" s="5">
-        <v>570</v>
+        <v>29</v>
+      </c>
+      <c r="C34" s="7">
+        <v>236</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="4">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C35" s="5">
-        <v>3912</v>
+        <v>29</v>
+      </c>
+      <c r="C35" s="7">
+        <v>4198</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C36" s="5">
-        <v>2398</v>
+      <c r="C36" s="7">
+        <v>224.2</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="4">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C37" s="5">
-        <v>590</v>
+      <c r="C37" s="7">
+        <v>5691</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C38" s="7">
-        <v>4300</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C39" s="7">
-        <v>236</v>
+        <v>4030</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="4">
-        <v>46196</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C40" s="7">
-        <v>4198</v>
-      </c>
+      <c r="A40" s="1"/>
+      <c r="B40" s="1"/>
+      <c r="C40" s="7"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="4">
-        <v>46196</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C41" s="7">
-        <v>224.2</v>
-      </c>
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="7"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="4">
-        <v>46196</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C42" s="7">
-        <v>5691</v>
-      </c>
+      <c r="A42" s="1"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="7"/>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="4">
-        <v>46197</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C43" s="7">
-        <v>4000</v>
-      </c>
+      <c r="A43" s="1"/>
+      <c r="B43" s="1"/>
+      <c r="C43" s="7"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="4">
-        <v>46197</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C44" s="7">
-        <v>4030</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="1"/>
-      <c r="B45" s="1"/>
-      <c r="C45" s="7"/>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="1"/>
-      <c r="B46" s="1"/>
-      <c r="C46" s="7"/>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="1"/>
-      <c r="B47" s="1"/>
-      <c r="C47" s="7"/>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="1"/>
-      <c r="B48" s="1"/>
-      <c r="C48" s="7"/>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="1"/>
-      <c r="B49" s="1"/>
-      <c r="C49" s="7"/>
+      <c r="A44" s="1"/>
+      <c r="B44" s="1"/>
+      <c r="C44" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1113,7 +1055,7 @@
         <v>46178</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C3" s="1">
         <v>280.23</v>
@@ -1124,7 +1066,7 @@
         <v>46191</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C4" s="8">
         <v>6018</v>
@@ -1729,7 +1671,7 @@
         <v>46179</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C28" s="7">
         <v>12</v>
@@ -1740,7 +1682,7 @@
         <v>46179</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C29" s="7">
         <v>67</v>
@@ -1751,7 +1693,7 @@
         <v>46179</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C30" s="7">
         <v>1</v>
@@ -1762,7 +1704,7 @@
         <v>46180</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C31" s="7">
         <v>57</v>
@@ -1773,7 +1715,7 @@
         <v>46180</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C32" s="7">
         <v>1.5</v>
@@ -1795,7 +1737,7 @@
         <v>46182</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C34" s="7">
         <v>78</v>
@@ -1806,7 +1748,7 @@
         <v>46183</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C35" s="7">
         <v>32.75</v>
@@ -1817,7 +1759,7 @@
         <v>46183</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C36" s="7">
         <v>39</v>
@@ -1828,7 +1770,7 @@
         <v>46192</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C37" s="7">
         <v>450.45</v>

</xml_diff>